<commit_message>
Add regtab stats/relabel/mixed model support and expand QA tests
</commit_message>
<xml_diff>
--- a/tabtools/demo/tablex.xlsx
+++ b/tabtools/demo/tablex.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="30" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="90" uniqueCount="18">
   <si>
     <t>Table 4. Summary by Origin</t>
   </si>
@@ -73,10 +73,974 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="114">
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
+  <fonts count="340">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="11"/>
@@ -569,7 +1533,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="80">
+  <borders count="238">
     <border>
       <left/>
       <right/>
@@ -1106,11 +2070,1069 @@
       <bottom style="thin"/>
       <diagonal style="none"/>
     </border>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="238">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
@@ -1413,6 +3435,614 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="113" fillId="0" borderId="79" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="80" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="81" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="82" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="83" xfId="0"/>
+    <xf numFmtId="0" fontId="114" fillId="0" borderId="84" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="115" fillId="0" borderId="85" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="116" fillId="0" borderId="86" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="117" fillId="0" borderId="87" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="118" fillId="0" borderId="88" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="119" fillId="0" borderId="89" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="120" fillId="0" borderId="90" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="121" fillId="0" borderId="91" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="122" fillId="0" borderId="92" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="123" fillId="0" borderId="93" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="125" fillId="0" borderId="94" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="127" fillId="0" borderId="95" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="129" fillId="0" borderId="96" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="131" fillId="0" borderId="97" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="133" fillId="0" borderId="98" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="135" fillId="0" borderId="99" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="137" fillId="0" borderId="100" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="139" fillId="0" borderId="101" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="141" fillId="0" borderId="102" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="143" fillId="0" borderId="103" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="144" fillId="0" borderId="104" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="145" fillId="0" borderId="105" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="146" fillId="0" borderId="106" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="147" fillId="0" borderId="107" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="148" fillId="0" borderId="108" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="150" fillId="0" borderId="109" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="152" fillId="0" borderId="110" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="154" fillId="0" borderId="111" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="156" fillId="0" borderId="112" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="158" fillId="0" borderId="113" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="160" fillId="0" borderId="114" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="162" fillId="0" borderId="115" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="164" fillId="0" borderId="116" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="166" fillId="0" borderId="117" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="168" fillId="0" borderId="118" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="170" fillId="0" borderId="119" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="172" fillId="0" borderId="120" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="174" fillId="0" borderId="121" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="176" fillId="0" borderId="122" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="178" fillId="0" borderId="123" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="180" fillId="0" borderId="124" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="181" fillId="0" borderId="125" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="182" fillId="0" borderId="126" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="183" fillId="0" borderId="127" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="184" fillId="0" borderId="128" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="185" fillId="0" borderId="129" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="186" fillId="0" borderId="130" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="187" fillId="0" borderId="131" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="188" fillId="0" borderId="132" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="189" fillId="0" borderId="133" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="190" fillId="0" borderId="134" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="191" fillId="0" borderId="135" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="192" fillId="0" borderId="136" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="193" fillId="0" borderId="137" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="194" fillId="0" borderId="138" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="195" fillId="0" borderId="139" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="196" fillId="0" borderId="140" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="197" fillId="0" borderId="141" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="198" fillId="0" borderId="142" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="199" fillId="0" borderId="143" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="200" fillId="0" borderId="144" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="201" fillId="0" borderId="145" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="202" fillId="0" borderId="146" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="204" fillId="0" borderId="147" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="206" fillId="0" borderId="148" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="208" fillId="0" borderId="149" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="210" fillId="0" borderId="150" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="212" fillId="0" borderId="151" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="214" fillId="0" borderId="152" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="216" fillId="0" borderId="153" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="218" fillId="0" borderId="154" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="220" fillId="0" borderId="155" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="222" fillId="0" borderId="156" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="224" fillId="0" borderId="157" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="226" fillId="0" borderId="158" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="159" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="160" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="161" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="162" xfId="0"/>
+    <xf numFmtId="0" fontId="227" fillId="0" borderId="163" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="228" fillId="0" borderId="164" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="229" fillId="0" borderId="165" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="230" fillId="0" borderId="166" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="231" fillId="0" borderId="167" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="232" fillId="0" borderId="168" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="233" fillId="0" borderId="169" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="234" fillId="0" borderId="170" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="235" fillId="0" borderId="171" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="236" fillId="0" borderId="172" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="238" fillId="0" borderId="173" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="240" fillId="0" borderId="174" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="242" fillId="0" borderId="175" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="244" fillId="0" borderId="176" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="246" fillId="0" borderId="177" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="248" fillId="0" borderId="178" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="250" fillId="0" borderId="179" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="252" fillId="0" borderId="180" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="254" fillId="0" borderId="181" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="256" fillId="0" borderId="182" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="257" fillId="0" borderId="183" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="258" fillId="0" borderId="184" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="259" fillId="0" borderId="185" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="260" fillId="0" borderId="186" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="261" fillId="0" borderId="187" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="263" fillId="0" borderId="188" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="265" fillId="0" borderId="189" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="267" fillId="0" borderId="190" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="269" fillId="0" borderId="191" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="271" fillId="0" borderId="192" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="273" fillId="0" borderId="193" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="275" fillId="0" borderId="194" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="277" fillId="0" borderId="195" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="279" fillId="0" borderId="196" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="281" fillId="0" borderId="197" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="283" fillId="0" borderId="198" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="285" fillId="0" borderId="199" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="287" fillId="0" borderId="200" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="289" fillId="0" borderId="201" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="291" fillId="0" borderId="202" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="293" fillId="0" borderId="203" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="294" fillId="0" borderId="204" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="295" fillId="0" borderId="205" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="296" fillId="0" borderId="206" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="297" fillId="0" borderId="207" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="298" fillId="0" borderId="208" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="299" fillId="0" borderId="209" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="300" fillId="0" borderId="210" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="301" fillId="0" borderId="211" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="302" fillId="0" borderId="212" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="303" fillId="0" borderId="213" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="304" fillId="0" borderId="214" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="305" fillId="0" borderId="215" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="306" fillId="0" borderId="216" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="307" fillId="0" borderId="217" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="308" fillId="0" borderId="218" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="309" fillId="0" borderId="219" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="310" fillId="0" borderId="220" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="311" fillId="0" borderId="221" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="312" fillId="0" borderId="222" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="313" fillId="0" borderId="223" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="314" fillId="0" borderId="224" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="315" fillId="0" borderId="225" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="317" fillId="0" borderId="226" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="319" fillId="0" borderId="227" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="321" fillId="0" borderId="228" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="323" fillId="0" borderId="229" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="325" fillId="0" borderId="230" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="327" fillId="0" borderId="231" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="329" fillId="0" borderId="232" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="331" fillId="0" borderId="233" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="333" fillId="0" borderId="234" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="335" fillId="0" borderId="235" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="337" fillId="0" borderId="236" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="339" fillId="0" borderId="237" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1428,110 +4058,110 @@
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" style="2" customWidth="true"/>
-    <col min="2" max="2" width="12.7109375" style="3" customWidth="true"/>
-    <col min="3" max="5" width="15.7109375" style="4" customWidth="true"/>
+    <col min="1" max="1" width="2.7109375" style="160" customWidth="true"/>
+    <col min="2" max="2" width="12.7109375" style="161" customWidth="true"/>
+    <col min="3" max="5" width="15.7109375" style="162" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="true" ht="30" customHeight="true">
-      <c r="A1" s="25" t="s">
+    <row r="1" s="159" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="183" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="183" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="183" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="D1" s="183" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="E1" s="183" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
+      <c r="A2" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="212" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="47" t="s">
+      <c r="C2" s="205" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="206" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="59" t="s">
+      <c r="E2" s="217" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s">
+      <c r="A3" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="55" t="s">
+      <c r="B3" s="213" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="51" t="s">
+      <c r="C3" s="209" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="52" t="s">
+      <c r="D3" s="210" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="60" t="s">
+      <c r="E3" s="218" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s">
+      <c r="A4" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="68" t="s">
+      <c r="B4" s="226" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="69" t="s">
+      <c r="C4" s="227" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="70" t="s">
+      <c r="D4" s="228" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="71" t="s">
+      <c r="E4" s="229" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="s">
+      <c r="A5" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="72" t="s">
+      <c r="B5" s="230" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="73" t="s">
+      <c r="C5" s="231" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="74" t="s">
+      <c r="D5" s="232" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="75" t="s">
+      <c r="E5" s="233" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="s">
+      <c r="A6" s="81" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="76" t="s">
+      <c r="B6" s="234" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="77" t="s">
+      <c r="C6" s="235" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="78" t="s">
+      <c r="D6" s="236" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="79" t="s">
+      <c r="E6" s="237" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>